<commit_message>
Remove unused categories and align taxonomy with seeded posts.
Drop 基礎知識, 飲食保健, and 健檢判讀 so only the five client-assigned categories are seeded, fixing homepage category nav validation and keeping copy and xlsx options in sync.
</commit_message>
<xml_diff>
--- a/materials/文章分類確認.xlsx
+++ b/materials/文章分類確認.xlsx
@@ -533,6 +533,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -565,7 +566,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>基礎知識、胰臟癌、胰臟發炎、胰臟水泡、飲食保健、健檢判讀</t>
+          <t>胰臟癌、胰臟癌篩檢、胰臟健康、胰臟發炎、胰臟水泡</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
@@ -7359,12 +7360,12 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>基礎知識</t>
+          <t>胰臟癌</t>
         </is>
       </c>
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>用白話方式介紹胰臟功能、常見症狀與就醫時機。</t>
+          <t>風險因子、早期警訊、篩檢策略與治療追蹤。</t>
         </is>
       </c>
       <c r="C2" s="13" t="n"/>
@@ -7395,34 +7396,38 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>胰臟癌</t>
+          <t>胰臟癌篩檢</t>
         </is>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>風險因子、早期警訊、篩檢策略與治療追蹤。</t>
+          <t>整理胰臟癌高風險族群的篩檢策略、追蹤時機與早期攔截方法。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>胰臟發炎</t>
+          <t>胰臟健康</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>急性與慢性胰臟炎、誘發因素與日常管理。</t>
+          <t>飲食原則與生活型態，從日常守護胰臟。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>胰臟癌篩檢</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="n"/>
+          <t>胰臟發炎</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>急性與慢性胰臟炎、誘發因素與日常管理。</t>
+        </is>
+      </c>
       <c r="C5" s="19" t="n"/>
       <c r="D5" s="19" t="n"/>
       <c r="E5" s="19" t="n"/>
@@ -7449,8 +7454,16 @@
       <c r="Z5" s="19" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="n"/>
-      <c r="B6" s="18" t="n"/>
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>胰臟水泡</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>囊腫與水泡類型、追蹤與需進一步評估的發現。</t>
+        </is>
+      </c>
       <c r="C6" s="18" t="n"/>
       <c r="D6" s="18" t="n"/>
       <c r="E6" s="18" t="n"/>
@@ -7477,16 +7490,8 @@
       <c r="Z6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>胰臟水泡</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>囊腫與水泡類型、追蹤與需進一步評估的發現。</t>
-        </is>
-      </c>
+      <c r="A7" s="18" t="n"/>
+      <c r="B7" s="18" t="n"/>
       <c r="C7" s="18" t="n"/>
       <c r="D7" s="18" t="n"/>
       <c r="E7" s="18" t="n"/>
@@ -7513,21 +7518,9 @@
       <c r="Z7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>胰臟健康</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>飲食原則與生活型態</t>
-        </is>
-      </c>
-      <c r="C8" s="26" t="inlineStr">
-        <is>
-          <t>胰臟功能</t>
-        </is>
-      </c>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="19" t="n"/>
+      <c r="C8" s="26" t="n"/>
       <c r="D8" s="12" t="inlineStr">
         <is>
           <t>飲食保健</t>
@@ -7589,16 +7582,8 @@
       <c r="Z9" s="19" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>飲食保健</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>飲食原則與生活型態，從日常守護胰臟。</t>
-        </is>
-      </c>
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="12" t="n"/>
       <c r="C10" s="12" t="n"/>
       <c r="D10" s="12" t="n"/>
       <c r="E10" s="12" t="n"/>
@@ -7625,16 +7610,8 @@
       <c r="Z10" s="12" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>健檢判讀</t>
-        </is>
-      </c>
-      <c r="B11" s="21" t="inlineStr">
-        <is>
-          <t>影像與血液檢查結果、報告用語解讀。</t>
-        </is>
-      </c>
+      <c r="A11" s="21" t="n"/>
+      <c r="B11" s="21" t="n"/>
       <c r="C11" s="21" t="n"/>
       <c r="D11" s="21" t="n"/>
       <c r="E11" s="21" t="n"/>
@@ -7661,11 +7638,7 @@
       <c r="Z11" s="21" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
-        <is>
-          <t>胰臟功能</t>
-        </is>
-      </c>
+      <c r="A12" s="22" t="n"/>
       <c r="B12" s="12" t="n"/>
       <c r="C12" s="12" t="n"/>
       <c r="D12" s="12" t="n"/>

</xml_diff>